<commit_message>
2026-06-22 15:40 fixing issues with latest data dictionary changes
</commit_message>
<xml_diff>
--- a/inst/cprd/hes_ae.xlsx
+++ b/inst/cprd/hes_ae.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="99">
   <si>
     <t xml:space="preserve">Column name</t>
   </si>
@@ -63,7 +63,7 @@
     <t xml:space="preserve">5</t>
   </si>
   <si>
-    <t xml:space="preserve">gen_hesid</t>
+    <t xml:space="preserve">cprd_mpsid</t>
   </si>
   <si>
     <t xml:space="preserve">A generated unique key assigned to a patient across all
@@ -73,20 +73,6 @@
 change between linkage sets.</t>
   </si>
   <si>
-    <t xml:space="preserve">n_patid_hes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Number of individuals in CPRD GOLD or CPRD Aurum
-assigned the same gen_hesid (unique patient identifier
-generated in HES)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INTEGER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
     <t xml:space="preserve">gen_ethnicity</t>
   </si>
   <si>
@@ -98,18 +84,6 @@
     <t xml:space="preserve">10</t>
   </si>
   <si>
-    <t xml:space="preserve">match_rank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indicates the quality of matching between a record in HES
-and CPRD primary care data and gives the level of
-confidence that an HES record has been correctly
-matched to a patient in CPRD GOLD or CPRD Aurum.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Encrypted unique key given to a patient in CPRD
 GOLD or CPRD Aurum [primary key, in combination
 with aekey]</t>
@@ -140,6 +114,9 @@
     <t xml:space="preserve">The reason for an A&amp;E episode</t>
   </si>
   <si>
+    <t xml:space="preserve">INTEGER</t>
+  </si>
+  <si>
     <t xml:space="preserve">2</t>
   </si>
   <si>
@@ -149,6 +126,9 @@
     <t xml:space="preserve">An indication of whether a patient is making an initial
 or follow-up attendance within a particular A&amp;E
 department</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
   </si>
   <si>
     <t xml:space="preserve">aearrivalmode</t>
@@ -257,6 +237,9 @@
 code. If no sub-analysis has been provided, or is not
 applicable, then the 2-character description is displayed if
 available.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
   </si>
   <si>
     <t xml:space="preserve">diaga</t>
@@ -736,40 +719,14 @@
         <v>14</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
+    </row>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -814,7 +771,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
@@ -825,10 +782,10 @@
     </row>
     <row r="3" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -839,184 +796,184 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="105.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1062,7 +1019,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
@@ -1073,10 +1030,10 @@
     </row>
     <row r="3" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -1087,100 +1044,100 @@
     </row>
     <row r="4" customFormat="false" ht="120.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="150.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1225,7 +1182,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
@@ -1236,10 +1193,10 @@
     </row>
     <row r="3" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -1250,44 +1207,44 @@
     </row>
     <row r="4" customFormat="false" ht="240.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="195.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1332,7 +1289,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
@@ -1343,10 +1300,10 @@
     </row>
     <row r="3" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -1357,58 +1314,58 @@
     </row>
     <row r="4" customFormat="false" ht="285.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="195.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="479.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1454,7 +1411,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
@@ -1465,10 +1422,10 @@
     </row>
     <row r="3" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -1479,72 +1436,72 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>16</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="165.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1589,7 +1546,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
@@ -1600,10 +1557,10 @@
     </row>
     <row r="3" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -1614,30 +1571,30 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>